<commit_message>
additional response equipment information
</commit_message>
<xml_diff>
--- a/docs/SLMS2026_import_cai_tao_bo_sung.xlsx
+++ b/docs/SLMS2026_import_cai_tao_bo_sung.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <cols>
     <col min="1" max="1" width="43.83203125" customWidth="1"/>
   </cols>
@@ -432,12 +432,12 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Sheet "1. Hop_Dong_Cai_Tao": chi phí cải tạo đợt này (gắn session hiện tại).</v>
+        <v>Sheet "1. Hop_Dong_Cai_Tao": chi phí cải tạo đợt này.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Sheet "2. Thiet_Bi_Mua_Moi": TB mua — THEM_MOI giữ TB cũ; THAY_THE disable TB ACTIVE cùng vị trí + catalog.</v>
+        <v>Sheet "2. Thiet_Bi_Mua_Moi": THEM_MOI giữ TB cũ; THAY_THE disable TB ACTIVE cùng vị trí + catalog.</v>
       </c>
     </row>
     <row r="8">
@@ -445,9 +445,14 @@
         <v>KHÔNG có sheet cấu hình khai thác / danh sách phòng.</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Mẫu: 5 dòng cải tạo, 6 dòng TB (4 HĐ).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -712,7 +717,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E6"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="23.83203125" customWidth="1"/>
@@ -772,16 +777,67 @@
         <v>Thay router WiFi toàn nhà</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>HD-WH-RENO-SPLIT</v>
+      </c>
+      <c r="B4" t="str">
+        <v>PLUMBING</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Điện nước</v>
+      </c>
+      <c r="D4">
+        <v>6000000</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Sửa rò rỉ phòng 102</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>HD-WH-RENO-SPLIT8</v>
+      </c>
+      <c r="B5" t="str">
+        <v>OTHER</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Khác</v>
+      </c>
+      <c r="D5">
+        <v>4000000</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Lắp camera an ninh</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>HD-WH-RENO-HANOI</v>
+      </c>
+      <c r="B6" t="str">
+        <v>FLOORING</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Sàn nhà</v>
+      </c>
+      <c r="D6">
+        <v>18000000</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Thay sàn gỗ phòng master</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L7"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -870,7 +926,7 @@
         <v>2030-12-31</v>
       </c>
       <c r="L2" t="str">
-        <v>Thay điều hòa mới phòng khách (disable bản v1)</v>
+        <v>Thay điều hòa mới phòng khách</v>
       </c>
     </row>
     <row r="3">
@@ -908,12 +964,164 @@
         <v>2027-12-31</v>
       </c>
       <c r="L3" t="str">
-        <v>Thêm quạt trần — giữ nguyên đồ cũ</v>
+        <v>Thêm quạt trần — giữ đồ cũ</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>HD-WH-RENO-SPLIT</v>
+      </c>
+      <c r="B4" t="str">
+        <v>102</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>Điều hòa</v>
+      </c>
+      <c r="E4" t="str">
+        <v>NEW</v>
+      </c>
+      <c r="F4" t="str">
+        <v>THAY_THE</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>9500000</v>
+      </c>
+      <c r="I4">
+        <v>24</v>
+      </c>
+      <c r="J4" t="str">
+        <v>2027-03-01</v>
+      </c>
+      <c r="K4" t="str">
+        <v>2029-02-28</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Thay điều hòa phòng 102</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>HD-WH-RENO-SPLIT</v>
+      </c>
+      <c r="B5" t="str">
+        <v>103</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>Giường</v>
+      </c>
+      <c r="E5" t="str">
+        <v>NEW</v>
+      </c>
+      <c r="F5" t="str">
+        <v>THEM_MOI</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>4500000</v>
+      </c>
+      <c r="I5">
+        <v>12</v>
+      </c>
+      <c r="J5" t="str">
+        <v>2027-03-01</v>
+      </c>
+      <c r="K5" t="str">
+        <v>2028-02-28</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Thêm giường tầng phòng 103</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>HD-WH-RENO-SPLIT8</v>
+      </c>
+      <c r="B6" t="str">
+        <v>105</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v>Nóng lạnh</v>
+      </c>
+      <c r="E6" t="str">
+        <v>NEW</v>
+      </c>
+      <c r="F6" t="str">
+        <v>THEM_MOI</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>2600000</v>
+      </c>
+      <c r="I6">
+        <v>12</v>
+      </c>
+      <c r="J6" t="str">
+        <v>2027-06-01</v>
+      </c>
+      <c r="K6" t="str">
+        <v>2028-05-31</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Lắp nóng lạnh phòng 105</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>HD-WH-RENO-HANOI</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v>KITCHEN</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Tủ lạnh</v>
+      </c>
+      <c r="E7" t="str">
+        <v>NEW</v>
+      </c>
+      <c r="F7" t="str">
+        <v>THAY_THE</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>22000000</v>
+      </c>
+      <c r="I7">
+        <v>36</v>
+      </c>
+      <c r="J7" t="str">
+        <v>2027-08-01</v>
+      </c>
+      <c r="K7" t="str">
+        <v>2030-07-31</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Thay tủ lạnh lớn hơn</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>